<commit_message>
feat: update data to Apr 2026 + add minutes bar data + fix deprecation
- Replace spot CSV with latest data (D_37090, through Mar 2026)
- Update 2026/2027 term structure CSVs with latest closes
- Update S&D Excels with Feb 2026 data
- Add fcpo_daily_term_delta.xlsx export
- Add Raw Data/Minutes Data/ (1-min bars per contract, 2024–2027)
- FCPO_analysis.py: auto-detect spot CSV; handle ISO + Unix timestamps
- app.py: remove deprecated infer_datetime_format=True in load_contracts()

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Raw Data/Stock and Production/FCPO Stock 3Y.xlsx
+++ b/Raw Data/Stock and Production/FCPO Stock 3Y.xlsx
@@ -1,42 +1,47 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr codeName="ThisWorkbook"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ClaudeCode\Raw Data\Stock and Production\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8D31C48-8EC0-46B8-9E02-A87DB23C92D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="40350" yWindow="1950" windowWidth="28800" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
     <sheet name="Table Data" sheetId="1" r:id="rId1"/>
   </sheets>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
-<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
-  <metadataTypes count="1">
-    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
-  </metadataTypes>
-  <futureMetadata name="XLDAPR" count="1">
-    <bk>
-      <extLst>
-        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
-          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
-        </ext>
-      </extLst>
-    </bk>
-  </futureMetadata>
-  <cellMetadata count="1">
-    <bk>
-      <rc t="1" v="0"/>
-    </bk>
-  </cellMetadata>
-</metadata>
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+  <si>
+    <t>Date</t>
+  </si>
+  <si>
+    <t>MYPOMS-TPO (COMM_LAST)</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>Close</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="2">
-    <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
-    <numFmt numFmtId="60" formatCode="dd/M/yyyy;@"/>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="dd/m/yyyy;@"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -66,14 +71,22 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="60" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -398,328 +411,338 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B39"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:B40"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.83203125" customWidth="1"/>
-    <col min="2" max="2" width="24.83203125" customWidth="1"/>
+    <col min="1" max="1" width="11.875" customWidth="1"/>
+    <col min="2" max="2" width="24.875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>Date</v>
-      </c>
-      <c r="B1" t="str">
-        <v>MYPOMS-TPO (COMM_LAST)</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v/>
-      </c>
-      <c r="B2" t="str">
-        <v>Close</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="1" t="d">
-        <v>2026-01-01T00:00:00.000Z</v>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" s="1">
+        <v>46054</v>
       </c>
       <c r="B3">
+        <v>2704286</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" s="1">
+        <v>46023</v>
+      </c>
+      <c r="B4">
         <v>2815493</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="1" t="d">
-        <v>2025-12-01T00:00:00.000Z</v>
-      </c>
-      <c r="B4">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" s="1">
+        <v>45992</v>
+      </c>
+      <c r="B5">
         <v>3051147</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="1" t="d">
-        <v>2025-11-01T00:00:00.000Z</v>
-      </c>
-      <c r="B5">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" s="1">
+        <v>45962</v>
+      </c>
+      <c r="B6">
         <v>2835578</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="1" t="d">
-        <v>2025-10-01T00:00:00.000Z</v>
-      </c>
-      <c r="B6">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" s="1">
+        <v>45931</v>
+      </c>
+      <c r="B7">
         <v>2508396</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="1" t="d">
-        <v>2025-09-01T00:00:00.000Z</v>
-      </c>
-      <c r="B7">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" s="1">
+        <v>45901</v>
+      </c>
+      <c r="B8">
         <v>2359572</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="1" t="d">
-        <v>2025-08-01T00:00:00.000Z</v>
-      </c>
-      <c r="B8">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" s="1">
+        <v>45870</v>
+      </c>
+      <c r="B9">
         <v>2202413</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="1" t="d">
-        <v>2025-07-01T00:00:00.000Z</v>
-      </c>
-      <c r="B9">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" s="1">
+        <v>45839</v>
+      </c>
+      <c r="B10">
         <v>2114085</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="1" t="d">
-        <v>2025-06-01T00:00:00.000Z</v>
-      </c>
-      <c r="B10">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" s="1">
+        <v>45809</v>
+      </c>
+      <c r="B11">
         <v>2031560</v>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="1" t="d">
-        <v>2025-05-01T00:00:00.000Z</v>
-      </c>
-      <c r="B11">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" s="1">
+        <v>45778</v>
+      </c>
+      <c r="B12">
         <v>1982759</v>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="1" t="d">
-        <v>2025-04-01T00:00:00.000Z</v>
-      </c>
-      <c r="B12">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13" s="1">
+        <v>45748</v>
+      </c>
+      <c r="B13">
         <v>1866124</v>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="1" t="d">
-        <v>2025-03-01T00:00:00.000Z</v>
-      </c>
-      <c r="B13">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A14" s="1">
+        <v>45717</v>
+      </c>
+      <c r="B14">
         <v>1562817</v>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="1" t="d">
-        <v>2025-02-01T00:00:00.000Z</v>
-      </c>
-      <c r="B14">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A15" s="1">
+        <v>45689</v>
+      </c>
+      <c r="B15">
         <v>1509525</v>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="1" t="d">
-        <v>2025-01-01T00:00:00.000Z</v>
-      </c>
-      <c r="B15">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A16" s="1">
+        <v>45658</v>
+      </c>
+      <c r="B16">
         <v>1580252</v>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="1" t="d">
-        <v>2024-12-01T00:00:00.000Z</v>
-      </c>
-      <c r="B16">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" s="1">
+        <v>45627</v>
+      </c>
+      <c r="B17">
         <v>1708756</v>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="1" t="d">
-        <v>2024-11-01T00:00:00.000Z</v>
-      </c>
-      <c r="B17">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A18" s="1">
+        <v>45597</v>
+      </c>
+      <c r="B18">
         <v>1835641</v>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="1" t="d">
-        <v>2024-10-01T00:00:00.000Z</v>
-      </c>
-      <c r="B18">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A19" s="1">
+        <v>45566</v>
+      </c>
+      <c r="B19">
         <v>1885183</v>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="1" t="d">
-        <v>2024-09-01T00:00:00.000Z</v>
-      </c>
-      <c r="B19">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A20" s="1">
+        <v>45536</v>
+      </c>
+      <c r="B20">
         <v>2011768</v>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="1" t="d">
-        <v>2024-08-01T00:00:00.000Z</v>
-      </c>
-      <c r="B20">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A21" s="1">
+        <v>45505</v>
+      </c>
+      <c r="B21">
         <v>1883328</v>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="1" t="d">
-        <v>2024-07-01T00:00:00.000Z</v>
-      </c>
-      <c r="B21">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A22" s="1">
+        <v>45474</v>
+      </c>
+      <c r="B22">
         <v>1754384</v>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="1" t="d">
-        <v>2024-06-01T00:00:00.000Z</v>
-      </c>
-      <c r="B22">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A23" s="1">
+        <v>45444</v>
+      </c>
+      <c r="B23">
         <v>1831239</v>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="1" t="d">
-        <v>2024-05-01T00:00:00.000Z</v>
-      </c>
-      <c r="B23">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A24" s="1">
+        <v>45413</v>
+      </c>
+      <c r="B24">
         <v>1753211</v>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="1" t="d">
-        <v>2024-04-01T00:00:00.000Z</v>
-      </c>
-      <c r="B24">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A25" s="1">
+        <v>45383</v>
+      </c>
+      <c r="B25">
         <v>1744459</v>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="1" t="d">
-        <v>2024-03-01T00:00:00.000Z</v>
-      </c>
-      <c r="B25">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A26" s="1">
+        <v>45352</v>
+      </c>
+      <c r="B26">
         <v>1714973</v>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="1" t="d">
-        <v>2024-02-01T00:00:00.000Z</v>
-      </c>
-      <c r="B26">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A27" s="1">
+        <v>45323</v>
+      </c>
+      <c r="B27">
         <v>1919210</v>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="1" t="d">
-        <v>2024-01-01T00:00:00.000Z</v>
-      </c>
-      <c r="B27">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A28" s="1">
+        <v>45292</v>
+      </c>
+      <c r="B28">
         <v>2019781</v>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="1" t="d">
-        <v>2023-12-01T00:00:00.000Z</v>
-      </c>
-      <c r="B28">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A29" s="1">
+        <v>45261</v>
+      </c>
+      <c r="B29">
         <v>2291167</v>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="1" t="d">
-        <v>2023-11-01T00:00:00.000Z</v>
-      </c>
-      <c r="B29">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A30" s="1">
+        <v>45231</v>
+      </c>
+      <c r="B30">
         <v>2420398</v>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="1" t="d">
-        <v>2023-10-01T00:00:00.000Z</v>
-      </c>
-      <c r="B30">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A31" s="1">
+        <v>45200</v>
+      </c>
+      <c r="B31">
         <v>2448852</v>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="1" t="d">
-        <v>2023-09-01T00:00:00.000Z</v>
-      </c>
-      <c r="B31">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A32" s="1">
+        <v>45170</v>
+      </c>
+      <c r="B32">
         <v>2313569</v>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="1" t="d">
-        <v>2023-08-01T00:00:00.000Z</v>
-      </c>
-      <c r="B32">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A33" s="1">
+        <v>45139</v>
+      </c>
+      <c r="B33">
         <v>2110980</v>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="1" t="d">
-        <v>2023-07-01T00:00:00.000Z</v>
-      </c>
-      <c r="B33">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A34" s="1">
+        <v>45108</v>
+      </c>
+      <c r="B34">
         <v>1734157</v>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="1" t="d">
-        <v>2023-06-01T00:00:00.000Z</v>
-      </c>
-      <c r="B34">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A35" s="1">
+        <v>45078</v>
+      </c>
+      <c r="B35">
         <v>1720567</v>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="1" t="d">
-        <v>2023-05-01T00:00:00.000Z</v>
-      </c>
-      <c r="B35">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A36" s="1">
+        <v>45047</v>
+      </c>
+      <c r="B36">
         <v>1686782</v>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="1" t="d">
-        <v>2023-04-01T00:00:00.000Z</v>
-      </c>
-      <c r="B36">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A37" s="1">
+        <v>45017</v>
+      </c>
+      <c r="B37">
         <v>1497617</v>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="1" t="d">
-        <v>2023-03-01T00:00:00.000Z</v>
-      </c>
-      <c r="B37">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A38" s="1">
+        <v>44986</v>
+      </c>
+      <c r="B38">
         <v>1674022</v>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="1" t="d">
-        <v>2023-02-01T00:00:00.000Z</v>
-      </c>
-      <c r="B38">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A39" s="1">
+        <v>44958</v>
+      </c>
+      <c r="B39">
         <v>2119848</v>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="1" t="d">
-        <v>2023-01-01T00:00:00.000Z</v>
-      </c>
-      <c r="B39">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A40" s="1">
+        <v>44927</v>
+      </c>
+      <c r="B40">
         <v>2268198</v>
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B39"/>
+    <ignoredError sqref="A4:B40 A1:B2" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: update all raw data through Apr 2026 and add supporting scripts
- Refresh term structure CSVs for 2020–2027 contracts
- Update MPOB stock, exports, production Excel files
- Add fcpo_combined_hourly.xlsx and fcpo_daily_term_delta.xlsx
- Add daily_term_combiner.py and daily_term_delta.py helper scripts
- Add fcpo_enriched_dataset.xlsx
- Update devcontainer, config, backtest, and server-setup-guide

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Raw Data/Stock and Production/FCPO Stock 3Y.xlsx
+++ b/Raw Data/Stock and Production/FCPO Stock 3Y.xlsx
@@ -1,42 +1,47 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr codeName="ThisWorkbook"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ClaudeCode\Raw Data\Stock and Production\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8D31C48-8EC0-46B8-9E02-A87DB23C92D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="40350" yWindow="1950" windowWidth="28800" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
     <sheet name="Table Data" sheetId="1" r:id="rId1"/>
   </sheets>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
-<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
-  <metadataTypes count="1">
-    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
-  </metadataTypes>
-  <futureMetadata name="XLDAPR" count="1">
-    <bk>
-      <extLst>
-        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
-          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
-        </ext>
-      </extLst>
-    </bk>
-  </futureMetadata>
-  <cellMetadata count="1">
-    <bk>
-      <rc t="1" v="0"/>
-    </bk>
-  </cellMetadata>
-</metadata>
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+  <si>
+    <t>Date</t>
+  </si>
+  <si>
+    <t>MYPOMS-TPO (COMM_LAST)</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>Close</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="2">
-    <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
-    <numFmt numFmtId="60" formatCode="dd/M/yyyy;@"/>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="dd/m/yyyy;@"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -66,14 +71,22 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="60" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -398,328 +411,338 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B39"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:B40"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.83203125" customWidth="1"/>
-    <col min="2" max="2" width="24.83203125" customWidth="1"/>
+    <col min="1" max="1" width="11.875" customWidth="1"/>
+    <col min="2" max="2" width="24.875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>Date</v>
-      </c>
-      <c r="B1" t="str">
-        <v>MYPOMS-TPO (COMM_LAST)</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v/>
-      </c>
-      <c r="B2" t="str">
-        <v>Close</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="1" t="d">
-        <v>2026-01-01T00:00:00.000Z</v>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" s="1">
+        <v>46054</v>
       </c>
       <c r="B3">
+        <v>2704286</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" s="1">
+        <v>46023</v>
+      </c>
+      <c r="B4">
         <v>2815493</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="1" t="d">
-        <v>2025-12-01T00:00:00.000Z</v>
-      </c>
-      <c r="B4">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" s="1">
+        <v>45992</v>
+      </c>
+      <c r="B5">
         <v>3051147</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="1" t="d">
-        <v>2025-11-01T00:00:00.000Z</v>
-      </c>
-      <c r="B5">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" s="1">
+        <v>45962</v>
+      </c>
+      <c r="B6">
         <v>2835578</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="1" t="d">
-        <v>2025-10-01T00:00:00.000Z</v>
-      </c>
-      <c r="B6">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" s="1">
+        <v>45931</v>
+      </c>
+      <c r="B7">
         <v>2508396</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="1" t="d">
-        <v>2025-09-01T00:00:00.000Z</v>
-      </c>
-      <c r="B7">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" s="1">
+        <v>45901</v>
+      </c>
+      <c r="B8">
         <v>2359572</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="1" t="d">
-        <v>2025-08-01T00:00:00.000Z</v>
-      </c>
-      <c r="B8">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" s="1">
+        <v>45870</v>
+      </c>
+      <c r="B9">
         <v>2202413</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="1" t="d">
-        <v>2025-07-01T00:00:00.000Z</v>
-      </c>
-      <c r="B9">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" s="1">
+        <v>45839</v>
+      </c>
+      <c r="B10">
         <v>2114085</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="1" t="d">
-        <v>2025-06-01T00:00:00.000Z</v>
-      </c>
-      <c r="B10">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" s="1">
+        <v>45809</v>
+      </c>
+      <c r="B11">
         <v>2031560</v>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="1" t="d">
-        <v>2025-05-01T00:00:00.000Z</v>
-      </c>
-      <c r="B11">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" s="1">
+        <v>45778</v>
+      </c>
+      <c r="B12">
         <v>1982759</v>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="1" t="d">
-        <v>2025-04-01T00:00:00.000Z</v>
-      </c>
-      <c r="B12">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13" s="1">
+        <v>45748</v>
+      </c>
+      <c r="B13">
         <v>1866124</v>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="1" t="d">
-        <v>2025-03-01T00:00:00.000Z</v>
-      </c>
-      <c r="B13">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A14" s="1">
+        <v>45717</v>
+      </c>
+      <c r="B14">
         <v>1562817</v>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="1" t="d">
-        <v>2025-02-01T00:00:00.000Z</v>
-      </c>
-      <c r="B14">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A15" s="1">
+        <v>45689</v>
+      </c>
+      <c r="B15">
         <v>1509525</v>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="1" t="d">
-        <v>2025-01-01T00:00:00.000Z</v>
-      </c>
-      <c r="B15">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A16" s="1">
+        <v>45658</v>
+      </c>
+      <c r="B16">
         <v>1580252</v>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="1" t="d">
-        <v>2024-12-01T00:00:00.000Z</v>
-      </c>
-      <c r="B16">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" s="1">
+        <v>45627</v>
+      </c>
+      <c r="B17">
         <v>1708756</v>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="1" t="d">
-        <v>2024-11-01T00:00:00.000Z</v>
-      </c>
-      <c r="B17">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A18" s="1">
+        <v>45597</v>
+      </c>
+      <c r="B18">
         <v>1835641</v>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="1" t="d">
-        <v>2024-10-01T00:00:00.000Z</v>
-      </c>
-      <c r="B18">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A19" s="1">
+        <v>45566</v>
+      </c>
+      <c r="B19">
         <v>1885183</v>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="1" t="d">
-        <v>2024-09-01T00:00:00.000Z</v>
-      </c>
-      <c r="B19">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A20" s="1">
+        <v>45536</v>
+      </c>
+      <c r="B20">
         <v>2011768</v>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="1" t="d">
-        <v>2024-08-01T00:00:00.000Z</v>
-      </c>
-      <c r="B20">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A21" s="1">
+        <v>45505</v>
+      </c>
+      <c r="B21">
         <v>1883328</v>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="1" t="d">
-        <v>2024-07-01T00:00:00.000Z</v>
-      </c>
-      <c r="B21">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A22" s="1">
+        <v>45474</v>
+      </c>
+      <c r="B22">
         <v>1754384</v>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="1" t="d">
-        <v>2024-06-01T00:00:00.000Z</v>
-      </c>
-      <c r="B22">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A23" s="1">
+        <v>45444</v>
+      </c>
+      <c r="B23">
         <v>1831239</v>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="1" t="d">
-        <v>2024-05-01T00:00:00.000Z</v>
-      </c>
-      <c r="B23">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A24" s="1">
+        <v>45413</v>
+      </c>
+      <c r="B24">
         <v>1753211</v>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="1" t="d">
-        <v>2024-04-01T00:00:00.000Z</v>
-      </c>
-      <c r="B24">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A25" s="1">
+        <v>45383</v>
+      </c>
+      <c r="B25">
         <v>1744459</v>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="1" t="d">
-        <v>2024-03-01T00:00:00.000Z</v>
-      </c>
-      <c r="B25">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A26" s="1">
+        <v>45352</v>
+      </c>
+      <c r="B26">
         <v>1714973</v>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="1" t="d">
-        <v>2024-02-01T00:00:00.000Z</v>
-      </c>
-      <c r="B26">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A27" s="1">
+        <v>45323</v>
+      </c>
+      <c r="B27">
         <v>1919210</v>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="1" t="d">
-        <v>2024-01-01T00:00:00.000Z</v>
-      </c>
-      <c r="B27">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A28" s="1">
+        <v>45292</v>
+      </c>
+      <c r="B28">
         <v>2019781</v>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="1" t="d">
-        <v>2023-12-01T00:00:00.000Z</v>
-      </c>
-      <c r="B28">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A29" s="1">
+        <v>45261</v>
+      </c>
+      <c r="B29">
         <v>2291167</v>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="1" t="d">
-        <v>2023-11-01T00:00:00.000Z</v>
-      </c>
-      <c r="B29">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A30" s="1">
+        <v>45231</v>
+      </c>
+      <c r="B30">
         <v>2420398</v>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="1" t="d">
-        <v>2023-10-01T00:00:00.000Z</v>
-      </c>
-      <c r="B30">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A31" s="1">
+        <v>45200</v>
+      </c>
+      <c r="B31">
         <v>2448852</v>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="1" t="d">
-        <v>2023-09-01T00:00:00.000Z</v>
-      </c>
-      <c r="B31">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A32" s="1">
+        <v>45170</v>
+      </c>
+      <c r="B32">
         <v>2313569</v>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="1" t="d">
-        <v>2023-08-01T00:00:00.000Z</v>
-      </c>
-      <c r="B32">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A33" s="1">
+        <v>45139</v>
+      </c>
+      <c r="B33">
         <v>2110980</v>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="1" t="d">
-        <v>2023-07-01T00:00:00.000Z</v>
-      </c>
-      <c r="B33">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A34" s="1">
+        <v>45108</v>
+      </c>
+      <c r="B34">
         <v>1734157</v>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="1" t="d">
-        <v>2023-06-01T00:00:00.000Z</v>
-      </c>
-      <c r="B34">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A35" s="1">
+        <v>45078</v>
+      </c>
+      <c r="B35">
         <v>1720567</v>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="1" t="d">
-        <v>2023-05-01T00:00:00.000Z</v>
-      </c>
-      <c r="B35">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A36" s="1">
+        <v>45047</v>
+      </c>
+      <c r="B36">
         <v>1686782</v>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="1" t="d">
-        <v>2023-04-01T00:00:00.000Z</v>
-      </c>
-      <c r="B36">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A37" s="1">
+        <v>45017</v>
+      </c>
+      <c r="B37">
         <v>1497617</v>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="1" t="d">
-        <v>2023-03-01T00:00:00.000Z</v>
-      </c>
-      <c r="B37">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A38" s="1">
+        <v>44986</v>
+      </c>
+      <c r="B38">
         <v>1674022</v>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="1" t="d">
-        <v>2023-02-01T00:00:00.000Z</v>
-      </c>
-      <c r="B38">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A39" s="1">
+        <v>44958</v>
+      </c>
+      <c r="B39">
         <v>2119848</v>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="1" t="d">
-        <v>2023-01-01T00:00:00.000Z</v>
-      </c>
-      <c r="B39">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A40" s="1">
+        <v>44927</v>
+      </c>
+      <c r="B40">
         <v>2268198</v>
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B39"/>
+    <ignoredError sqref="A4:B40 A1:B2" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix: session_state data flow for S producer — top panel now reflects last form submit
- Top of Tab 7 reads s_producer_current/s_forward from st.session_state (set on submit)
- Falls back to last producer_log.csv entry, then MPOB if no session state
- Form submit stores result in session_state so three-source comparison updates immediately
- Also includes: implied_s_backsolve formula fix (12x scaling), regression date/filter fixes,
  producer hist-low/current/high inputs replacing slider, Tab 8 SharePoint wiring

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Raw Data/Stock and Production/FCPO Stock 3Y.xlsx
+++ b/Raw Data/Stock and Production/FCPO Stock 3Y.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ClaudeCode\Raw Data\Stock and Production\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8D31C48-8EC0-46B8-9E02-A87DB23C92D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CCA9003-D2CE-491C-88DF-15E112DD43CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="40350" yWindow="1950" windowWidth="28800" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Table Data" sheetId="1" r:id="rId1"/>
@@ -412,7 +412,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B40"/>
+  <dimension ref="A1:B125"/>
   <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.875" customWidth="1"/>
@@ -437,312 +437,992 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
-        <v>46054</v>
+        <v>46082</v>
       </c>
       <c r="B3">
-        <v>2704286</v>
+        <v>2267260</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
-        <v>46023</v>
+        <v>46054</v>
       </c>
       <c r="B4">
-        <v>2815493</v>
+        <v>2704286</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
-        <v>45992</v>
+        <v>46023</v>
       </c>
       <c r="B5">
-        <v>3051147</v>
+        <v>2815493</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
-        <v>45962</v>
+        <v>45992</v>
       </c>
       <c r="B6">
-        <v>2835578</v>
+        <v>3051147</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
-        <v>45931</v>
+        <v>45962</v>
       </c>
       <c r="B7">
-        <v>2508396</v>
+        <v>2835578</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
-        <v>45901</v>
+        <v>45931</v>
       </c>
       <c r="B8">
-        <v>2359572</v>
+        <v>2508396</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
-        <v>45870</v>
+        <v>45901</v>
       </c>
       <c r="B9">
-        <v>2202413</v>
+        <v>2359572</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
-        <v>45839</v>
+        <v>45870</v>
       </c>
       <c r="B10">
-        <v>2114085</v>
+        <v>2202413</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
-        <v>45809</v>
+        <v>45839</v>
       </c>
       <c r="B11">
-        <v>2031560</v>
+        <v>2114085</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
-        <v>45778</v>
+        <v>45809</v>
       </c>
       <c r="B12">
-        <v>1982759</v>
+        <v>2031560</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
-        <v>45748</v>
+        <v>45778</v>
       </c>
       <c r="B13">
-        <v>1866124</v>
+        <v>1982759</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
-        <v>45717</v>
+        <v>45748</v>
       </c>
       <c r="B14">
-        <v>1562817</v>
+        <v>1866124</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="1">
-        <v>45689</v>
+        <v>45717</v>
       </c>
       <c r="B15">
-        <v>1509525</v>
+        <v>1562817</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" s="1">
-        <v>45658</v>
+        <v>45689</v>
       </c>
       <c r="B16">
-        <v>1580252</v>
+        <v>1509525</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="1">
-        <v>45627</v>
+        <v>45658</v>
       </c>
       <c r="B17">
-        <v>1708756</v>
+        <v>1580252</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" s="1">
-        <v>45597</v>
+        <v>45627</v>
       </c>
       <c r="B18">
-        <v>1835641</v>
+        <v>1708756</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" s="1">
-        <v>45566</v>
+        <v>45597</v>
       </c>
       <c r="B19">
-        <v>1885183</v>
+        <v>1835641</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" s="1">
-        <v>45536</v>
+        <v>45566</v>
       </c>
       <c r="B20">
-        <v>2011768</v>
+        <v>1885183</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" s="1">
-        <v>45505</v>
+        <v>45536</v>
       </c>
       <c r="B21">
-        <v>1883328</v>
+        <v>2011768</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" s="1">
-        <v>45474</v>
+        <v>45505</v>
       </c>
       <c r="B22">
-        <v>1754384</v>
+        <v>1883328</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" s="1">
-        <v>45444</v>
+        <v>45474</v>
       </c>
       <c r="B23">
-        <v>1831239</v>
+        <v>1754384</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" s="1">
-        <v>45413</v>
+        <v>45444</v>
       </c>
       <c r="B24">
-        <v>1753211</v>
+        <v>1831239</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" s="1">
-        <v>45383</v>
+        <v>45413</v>
       </c>
       <c r="B25">
-        <v>1744459</v>
+        <v>1753211</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" s="1">
-        <v>45352</v>
+        <v>45383</v>
       </c>
       <c r="B26">
-        <v>1714973</v>
+        <v>1744459</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" s="1">
-        <v>45323</v>
+        <v>45352</v>
       </c>
       <c r="B27">
-        <v>1919210</v>
+        <v>1714973</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" s="1">
-        <v>45292</v>
+        <v>45323</v>
       </c>
       <c r="B28">
-        <v>2019781</v>
+        <v>1919210</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" s="1">
-        <v>45261</v>
+        <v>45292</v>
       </c>
       <c r="B29">
-        <v>2291167</v>
+        <v>2019781</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" s="1">
-        <v>45231</v>
+        <v>45261</v>
       </c>
       <c r="B30">
-        <v>2420398</v>
+        <v>2291167</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31" s="1">
-        <v>45200</v>
+        <v>45231</v>
       </c>
       <c r="B31">
-        <v>2448852</v>
+        <v>2420398</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32" s="1">
-        <v>45170</v>
+        <v>45200</v>
       </c>
       <c r="B32">
-        <v>2313569</v>
+        <v>2448852</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" s="1">
-        <v>45139</v>
+        <v>45170</v>
       </c>
       <c r="B33">
-        <v>2110980</v>
+        <v>2313569</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" s="1">
-        <v>45108</v>
+        <v>45139</v>
       </c>
       <c r="B34">
-        <v>1734157</v>
+        <v>2110980</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" s="1">
-        <v>45078</v>
+        <v>45108</v>
       </c>
       <c r="B35">
-        <v>1720567</v>
+        <v>1734157</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36" s="1">
-        <v>45047</v>
+        <v>45078</v>
       </c>
       <c r="B36">
-        <v>1686782</v>
+        <v>1720567</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37" s="1">
-        <v>45017</v>
+        <v>45047</v>
       </c>
       <c r="B37">
-        <v>1497617</v>
+        <v>1686782</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38" s="1">
-        <v>44986</v>
+        <v>45017</v>
       </c>
       <c r="B38">
-        <v>1674022</v>
+        <v>1497617</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" s="1">
-        <v>44958</v>
+        <v>44986</v>
       </c>
       <c r="B39">
-        <v>2119848</v>
+        <v>1674022</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" s="1">
+        <v>44958</v>
+      </c>
+      <c r="B40">
+        <v>2119848</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A41" s="1">
         <v>44927</v>
       </c>
-      <c r="B40">
+      <c r="B41">
         <v>2268198</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A42" s="1">
+        <v>44896</v>
+      </c>
+      <c r="B42">
+        <v>2196574</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A43" s="1">
+        <v>44866</v>
+      </c>
+      <c r="B43">
+        <v>2288471</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A44" s="1">
+        <v>44835</v>
+      </c>
+      <c r="B44">
+        <v>2408293</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A45" s="1">
+        <v>44805</v>
+      </c>
+      <c r="B45">
+        <v>2317020</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A46" s="1">
+        <v>44774</v>
+      </c>
+      <c r="B46">
+        <v>2094667</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A47" s="1">
+        <v>44743</v>
+      </c>
+      <c r="B47">
+        <v>1772804</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A48" s="1">
+        <v>44713</v>
+      </c>
+      <c r="B48">
+        <v>1645831</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A49" s="1">
+        <v>44682</v>
+      </c>
+      <c r="B49">
+        <v>1521826</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A50" s="1">
+        <v>44652</v>
+      </c>
+      <c r="B50">
+        <v>1641994</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A51" s="1">
+        <v>44621</v>
+      </c>
+      <c r="B51">
+        <v>1472810</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A52" s="1">
+        <v>44593</v>
+      </c>
+      <c r="B52">
+        <v>1518238</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A53" s="1">
+        <v>44562</v>
+      </c>
+      <c r="B53">
+        <v>1552414</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A54" s="1">
+        <v>44531</v>
+      </c>
+      <c r="B54">
+        <v>1583040</v>
+      </c>
+    </row>
+    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A55" s="1">
+        <v>44501</v>
+      </c>
+      <c r="B55">
+        <v>1816879</v>
+      </c>
+    </row>
+    <row r="56" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A56" s="1">
+        <v>44470</v>
+      </c>
+      <c r="B56">
+        <v>1834103</v>
+      </c>
+    </row>
+    <row r="57" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A57" s="1">
+        <v>44440</v>
+      </c>
+      <c r="B57">
+        <v>1746520</v>
+      </c>
+    </row>
+    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A58" s="1">
+        <v>44409</v>
+      </c>
+      <c r="B58">
+        <v>1877773</v>
+      </c>
+    </row>
+    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A59" s="1">
+        <v>44378</v>
+      </c>
+      <c r="B59">
+        <v>1496460</v>
+      </c>
+    </row>
+    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A60" s="1">
+        <v>44348</v>
+      </c>
+      <c r="B60">
+        <v>1613657</v>
+      </c>
+    </row>
+    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A61" s="1">
+        <v>44317</v>
+      </c>
+      <c r="B61">
+        <v>1568943</v>
+      </c>
+    </row>
+    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A62" s="1">
+        <v>44287</v>
+      </c>
+      <c r="B62">
+        <v>1545981</v>
+      </c>
+    </row>
+    <row r="63" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A63" s="1">
+        <v>44256</v>
+      </c>
+      <c r="B63">
+        <v>1445970</v>
+      </c>
+    </row>
+    <row r="64" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A64" s="1">
+        <v>44228</v>
+      </c>
+      <c r="B64">
+        <v>1300808</v>
+      </c>
+    </row>
+    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A65" s="1">
+        <v>44197</v>
+      </c>
+      <c r="B65">
+        <v>1324963</v>
+      </c>
+    </row>
+    <row r="66" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A66" s="1">
+        <v>44166</v>
+      </c>
+      <c r="B66">
+        <v>1265698</v>
+      </c>
+    </row>
+    <row r="67" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A67" s="1">
+        <v>44136</v>
+      </c>
+      <c r="B67">
+        <v>1564505</v>
+      </c>
+    </row>
+    <row r="68" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A68" s="1">
+        <v>44105</v>
+      </c>
+      <c r="B68">
+        <v>1573665</v>
+      </c>
+    </row>
+    <row r="69" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A69" s="1">
+        <v>44075</v>
+      </c>
+      <c r="B69">
+        <v>1722007</v>
+      </c>
+    </row>
+    <row r="70" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A70" s="1">
+        <v>44044</v>
+      </c>
+      <c r="B70">
+        <v>1699106</v>
+      </c>
+    </row>
+    <row r="71" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A71" s="1">
+        <v>44013</v>
+      </c>
+      <c r="B71">
+        <v>1698036</v>
+      </c>
+    </row>
+    <row r="72" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A72" s="1">
+        <v>43983</v>
+      </c>
+      <c r="B72">
+        <v>1898331</v>
+      </c>
+    </row>
+    <row r="73" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A73" s="1">
+        <v>43952</v>
+      </c>
+      <c r="B73">
+        <v>2029579</v>
+      </c>
+    </row>
+    <row r="74" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A74" s="1">
+        <v>43922</v>
+      </c>
+      <c r="B74">
+        <v>2044498</v>
+      </c>
+    </row>
+    <row r="75" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A75" s="1">
+        <v>43891</v>
+      </c>
+      <c r="B75">
+        <v>1729592</v>
+      </c>
+    </row>
+    <row r="76" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A76" s="1">
+        <v>43862</v>
+      </c>
+      <c r="B76">
+        <v>1700261</v>
+      </c>
+    </row>
+    <row r="77" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A77" s="1">
+        <v>43831</v>
+      </c>
+      <c r="B77">
+        <v>1755417</v>
+      </c>
+    </row>
+    <row r="78" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A78" s="1">
+        <v>43800</v>
+      </c>
+      <c r="B78">
+        <v>2007124</v>
+      </c>
+    </row>
+    <row r="79" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A79" s="1">
+        <v>43770</v>
+      </c>
+      <c r="B79">
+        <v>2255035</v>
+      </c>
+    </row>
+    <row r="80" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A80" s="1">
+        <v>43739</v>
+      </c>
+      <c r="B80">
+        <v>2351994</v>
+      </c>
+    </row>
+    <row r="81" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A81" s="1">
+        <v>43709</v>
+      </c>
+      <c r="B81">
+        <v>2448272</v>
+      </c>
+    </row>
+    <row r="82" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A82" s="1">
+        <v>43678</v>
+      </c>
+      <c r="B82">
+        <v>2251831</v>
+      </c>
+    </row>
+    <row r="83" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A83" s="1">
+        <v>43647</v>
+      </c>
+      <c r="B83">
+        <v>2378099</v>
+      </c>
+    </row>
+    <row r="84" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A84" s="1">
+        <v>43617</v>
+      </c>
+      <c r="B84">
+        <v>2410746</v>
+      </c>
+    </row>
+    <row r="85" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A85" s="1">
+        <v>43586</v>
+      </c>
+      <c r="B85">
+        <v>2447250</v>
+      </c>
+    </row>
+    <row r="86" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A86" s="1">
+        <v>43556</v>
+      </c>
+      <c r="B86">
+        <v>2729389</v>
+      </c>
+    </row>
+    <row r="87" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A87" s="1">
+        <v>43525</v>
+      </c>
+      <c r="B87">
+        <v>2922852</v>
+      </c>
+    </row>
+    <row r="88" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A88" s="1">
+        <v>43497</v>
+      </c>
+      <c r="B88">
+        <v>3059400</v>
+      </c>
+    </row>
+    <row r="89" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A89" s="1">
+        <v>43466</v>
+      </c>
+      <c r="B89">
+        <v>3005313</v>
+      </c>
+    </row>
+    <row r="90" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A90" s="1">
+        <v>43435</v>
+      </c>
+      <c r="B90">
+        <v>3215052</v>
+      </c>
+    </row>
+    <row r="91" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A91" s="1">
+        <v>43405</v>
+      </c>
+      <c r="B91">
+        <v>3007086</v>
+      </c>
+    </row>
+    <row r="92" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A92" s="1">
+        <v>43374</v>
+      </c>
+      <c r="B92">
+        <v>2722478</v>
+      </c>
+    </row>
+    <row r="93" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A93" s="1">
+        <v>43344</v>
+      </c>
+      <c r="B93">
+        <v>2529447</v>
+      </c>
+    </row>
+    <row r="94" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A94" s="1">
+        <v>43313</v>
+      </c>
+      <c r="B94">
+        <v>2054915</v>
+      </c>
+    </row>
+    <row r="95" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A95" s="1">
+        <v>43282</v>
+      </c>
+      <c r="B95">
+        <v>2214689</v>
+      </c>
+    </row>
+    <row r="96" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A96" s="1">
+        <v>43252</v>
+      </c>
+      <c r="B96">
+        <v>2188660</v>
+      </c>
+    </row>
+    <row r="97" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A97" s="1">
+        <v>43221</v>
+      </c>
+      <c r="B97">
+        <v>2170431</v>
+      </c>
+    </row>
+    <row r="98" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A98" s="1">
+        <v>43191</v>
+      </c>
+      <c r="B98">
+        <v>2181478</v>
+      </c>
+    </row>
+    <row r="99" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A99" s="1">
+        <v>43160</v>
+      </c>
+      <c r="B99">
+        <v>2323458</v>
+      </c>
+    </row>
+    <row r="100" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A100" s="1">
+        <v>43132</v>
+      </c>
+      <c r="B100">
+        <v>2478186</v>
+      </c>
+    </row>
+    <row r="101" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A101" s="1">
+        <v>43101</v>
+      </c>
+      <c r="B101">
+        <v>2547680</v>
+      </c>
+    </row>
+    <row r="102" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A102" s="1">
+        <v>43070</v>
+      </c>
+      <c r="B102">
+        <v>2732093</v>
+      </c>
+    </row>
+    <row r="103" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A103" s="1">
+        <v>43040</v>
+      </c>
+      <c r="B103">
+        <v>2553739</v>
+      </c>
+    </row>
+    <row r="104" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A104" s="1">
+        <v>43009</v>
+      </c>
+      <c r="B104">
+        <v>2203383</v>
+      </c>
+    </row>
+    <row r="105" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A105" s="1">
+        <v>42979</v>
+      </c>
+      <c r="B105">
+        <v>2020505</v>
+      </c>
+    </row>
+    <row r="106" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A106" s="1">
+        <v>42948</v>
+      </c>
+      <c r="B106">
+        <v>1942001</v>
+      </c>
+    </row>
+    <row r="107" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A107" s="1">
+        <v>42917</v>
+      </c>
+      <c r="B107">
+        <v>1785082</v>
+      </c>
+    </row>
+    <row r="108" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A108" s="1">
+        <v>42887</v>
+      </c>
+      <c r="B108">
+        <v>1527071</v>
+      </c>
+    </row>
+    <row r="109" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A109" s="1">
+        <v>42856</v>
+      </c>
+      <c r="B109">
+        <v>1557354</v>
+      </c>
+    </row>
+    <row r="110" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A110" s="1">
+        <v>42826</v>
+      </c>
+      <c r="B110">
+        <v>599894</v>
+      </c>
+    </row>
+    <row r="111" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A111" s="1">
+        <v>42795</v>
+      </c>
+      <c r="B111">
+        <v>1552988</v>
+      </c>
+    </row>
+    <row r="112" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A112" s="1">
+        <v>42767</v>
+      </c>
+      <c r="B112">
+        <v>1459265</v>
+      </c>
+    </row>
+    <row r="113" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A113" s="1">
+        <v>42736</v>
+      </c>
+      <c r="B113">
+        <v>1541082</v>
+      </c>
+    </row>
+    <row r="114" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A114" s="1">
+        <v>42705</v>
+      </c>
+      <c r="B114">
+        <v>1665388</v>
+      </c>
+    </row>
+    <row r="115" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A115" s="1">
+        <v>42675</v>
+      </c>
+      <c r="B115">
+        <v>1662811</v>
+      </c>
+    </row>
+    <row r="116" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A116" s="1">
+        <v>42644</v>
+      </c>
+      <c r="B116">
+        <v>1574288</v>
+      </c>
+    </row>
+    <row r="117" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A117" s="1">
+        <v>42614</v>
+      </c>
+      <c r="B117">
+        <v>1546413</v>
+      </c>
+    </row>
+    <row r="118" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A118" s="1">
+        <v>42583</v>
+      </c>
+      <c r="B118">
+        <v>1464080</v>
+      </c>
+    </row>
+    <row r="119" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A119" s="1">
+        <v>42552</v>
+      </c>
+      <c r="B119">
+        <v>1770083</v>
+      </c>
+    </row>
+    <row r="120" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A120" s="1">
+        <v>42522</v>
+      </c>
+      <c r="B120">
+        <v>1774624</v>
+      </c>
+    </row>
+    <row r="121" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A121" s="1">
+        <v>42491</v>
+      </c>
+      <c r="B121">
+        <v>1649858</v>
+      </c>
+    </row>
+    <row r="122" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A122" s="1">
+        <v>42461</v>
+      </c>
+      <c r="B122">
+        <v>1803894</v>
+      </c>
+    </row>
+    <row r="123" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A123" s="1">
+        <v>42430</v>
+      </c>
+      <c r="B123">
+        <v>1885630</v>
+      </c>
+    </row>
+    <row r="124" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A124" s="1">
+        <v>42401</v>
+      </c>
+      <c r="B124">
+        <v>2170341</v>
+      </c>
+    </row>
+    <row r="125" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A125" s="1">
+        <v>42370</v>
+      </c>
+      <c r="B125">
+        <v>2308582</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A4:B40 A1:B2" numberStoredAsText="1"/>
+    <ignoredError sqref="A5:B41 A1:B2" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
data: update all raw data files and add 2018-2019 term structure
- Update spot price, S&D (Stock, Production), and 2026-2027 term structure CSVs
- Add historical term structure data for 2018 and 2019
- Add ENSO data files
- Add FCPO_Curve_Input.xlsx
- Rename MPOB Exports 3Y → MPOB Export 3Y

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Raw Data/Stock and Production/FCPO Stock 3Y.xlsx
+++ b/Raw Data/Stock and Production/FCPO Stock 3Y.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ClaudeCode\Raw Data\Stock and Production\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CCA9003-D2CE-491C-88DF-15E112DD43CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{601910F9-B5DD-4732-ABAE-4E01B784015A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="39390" yWindow="-20835" windowWidth="28800" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Table Data" sheetId="1" r:id="rId1"/>
@@ -412,7 +412,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B125"/>
+  <dimension ref="A1:B126"/>
   <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.875" customWidth="1"/>
@@ -437,992 +437,1000 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
-        <v>46082</v>
+        <v>46113</v>
       </c>
       <c r="B3">
-        <v>2267260</v>
+        <v>2309474</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
-        <v>46054</v>
+        <v>46082</v>
       </c>
       <c r="B4">
-        <v>2704286</v>
+        <v>2270574</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
-        <v>46023</v>
+        <v>46054</v>
       </c>
       <c r="B5">
-        <v>2815493</v>
+        <v>2704286</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
-        <v>45992</v>
+        <v>46023</v>
       </c>
       <c r="B6">
-        <v>3051147</v>
+        <v>2815493</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
-        <v>45962</v>
+        <v>45992</v>
       </c>
       <c r="B7">
-        <v>2835578</v>
+        <v>3051147</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
-        <v>45931</v>
+        <v>45962</v>
       </c>
       <c r="B8">
-        <v>2508396</v>
+        <v>2835578</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
-        <v>45901</v>
+        <v>45931</v>
       </c>
       <c r="B9">
-        <v>2359572</v>
+        <v>2508396</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
-        <v>45870</v>
+        <v>45901</v>
       </c>
       <c r="B10">
-        <v>2202413</v>
+        <v>2359572</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
-        <v>45839</v>
+        <v>45870</v>
       </c>
       <c r="B11">
-        <v>2114085</v>
+        <v>2202413</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
-        <v>45809</v>
+        <v>45839</v>
       </c>
       <c r="B12">
-        <v>2031560</v>
+        <v>2114085</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
-        <v>45778</v>
+        <v>45809</v>
       </c>
       <c r="B13">
-        <v>1982759</v>
+        <v>2031560</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
-        <v>45748</v>
+        <v>45778</v>
       </c>
       <c r="B14">
-        <v>1866124</v>
+        <v>1982759</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="1">
-        <v>45717</v>
+        <v>45748</v>
       </c>
       <c r="B15">
-        <v>1562817</v>
+        <v>1866124</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" s="1">
-        <v>45689</v>
+        <v>45717</v>
       </c>
       <c r="B16">
-        <v>1509525</v>
+        <v>1562817</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="1">
-        <v>45658</v>
+        <v>45689</v>
       </c>
       <c r="B17">
-        <v>1580252</v>
+        <v>1509525</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" s="1">
-        <v>45627</v>
+        <v>45658</v>
       </c>
       <c r="B18">
-        <v>1708756</v>
+        <v>1580252</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" s="1">
-        <v>45597</v>
+        <v>45627</v>
       </c>
       <c r="B19">
-        <v>1835641</v>
+        <v>1708756</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" s="1">
-        <v>45566</v>
+        <v>45597</v>
       </c>
       <c r="B20">
-        <v>1885183</v>
+        <v>1835641</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" s="1">
-        <v>45536</v>
+        <v>45566</v>
       </c>
       <c r="B21">
-        <v>2011768</v>
+        <v>1885183</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" s="1">
-        <v>45505</v>
+        <v>45536</v>
       </c>
       <c r="B22">
-        <v>1883328</v>
+        <v>2011768</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" s="1">
-        <v>45474</v>
+        <v>45505</v>
       </c>
       <c r="B23">
-        <v>1754384</v>
+        <v>1883328</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" s="1">
-        <v>45444</v>
+        <v>45474</v>
       </c>
       <c r="B24">
-        <v>1831239</v>
+        <v>1754384</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" s="1">
-        <v>45413</v>
+        <v>45444</v>
       </c>
       <c r="B25">
-        <v>1753211</v>
+        <v>1831239</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" s="1">
-        <v>45383</v>
+        <v>45413</v>
       </c>
       <c r="B26">
-        <v>1744459</v>
+        <v>1753211</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" s="1">
-        <v>45352</v>
+        <v>45383</v>
       </c>
       <c r="B27">
-        <v>1714973</v>
+        <v>1744459</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" s="1">
-        <v>45323</v>
+        <v>45352</v>
       </c>
       <c r="B28">
-        <v>1919210</v>
+        <v>1714973</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" s="1">
-        <v>45292</v>
+        <v>45323</v>
       </c>
       <c r="B29">
-        <v>2019781</v>
+        <v>1919210</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" s="1">
-        <v>45261</v>
+        <v>45292</v>
       </c>
       <c r="B30">
-        <v>2291167</v>
+        <v>2019781</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31" s="1">
-        <v>45231</v>
+        <v>45261</v>
       </c>
       <c r="B31">
-        <v>2420398</v>
+        <v>2291167</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32" s="1">
-        <v>45200</v>
+        <v>45231</v>
       </c>
       <c r="B32">
-        <v>2448852</v>
+        <v>2420398</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" s="1">
-        <v>45170</v>
+        <v>45200</v>
       </c>
       <c r="B33">
-        <v>2313569</v>
+        <v>2448852</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" s="1">
-        <v>45139</v>
+        <v>45170</v>
       </c>
       <c r="B34">
-        <v>2110980</v>
+        <v>2313569</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" s="1">
-        <v>45108</v>
+        <v>45139</v>
       </c>
       <c r="B35">
-        <v>1734157</v>
+        <v>2110980</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36" s="1">
-        <v>45078</v>
+        <v>45108</v>
       </c>
       <c r="B36">
-        <v>1720567</v>
+        <v>1734157</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37" s="1">
-        <v>45047</v>
+        <v>45078</v>
       </c>
       <c r="B37">
-        <v>1686782</v>
+        <v>1720567</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38" s="1">
-        <v>45017</v>
+        <v>45047</v>
       </c>
       <c r="B38">
-        <v>1497617</v>
+        <v>1686782</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" s="1">
-        <v>44986</v>
+        <v>45017</v>
       </c>
       <c r="B39">
-        <v>1674022</v>
+        <v>1497617</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" s="1">
-        <v>44958</v>
+        <v>44986</v>
       </c>
       <c r="B40">
-        <v>2119848</v>
+        <v>1674022</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41" s="1">
-        <v>44927</v>
+        <v>44958</v>
       </c>
       <c r="B41">
-        <v>2268198</v>
+        <v>2119848</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A42" s="1">
-        <v>44896</v>
+        <v>44927</v>
       </c>
       <c r="B42">
-        <v>2196574</v>
+        <v>2268198</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A43" s="1">
-        <v>44866</v>
+        <v>44896</v>
       </c>
       <c r="B43">
-        <v>2288471</v>
+        <v>2196574</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A44" s="1">
-        <v>44835</v>
+        <v>44866</v>
       </c>
       <c r="B44">
-        <v>2408293</v>
+        <v>2288471</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A45" s="1">
-        <v>44805</v>
+        <v>44835</v>
       </c>
       <c r="B45">
-        <v>2317020</v>
+        <v>2408293</v>
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A46" s="1">
-        <v>44774</v>
+        <v>44805</v>
       </c>
       <c r="B46">
-        <v>2094667</v>
+        <v>2317020</v>
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A47" s="1">
-        <v>44743</v>
+        <v>44774</v>
       </c>
       <c r="B47">
-        <v>1772804</v>
+        <v>2094667</v>
       </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A48" s="1">
-        <v>44713</v>
+        <v>44743</v>
       </c>
       <c r="B48">
-        <v>1645831</v>
+        <v>1772804</v>
       </c>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A49" s="1">
-        <v>44682</v>
+        <v>44713</v>
       </c>
       <c r="B49">
-        <v>1521826</v>
+        <v>1645831</v>
       </c>
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A50" s="1">
-        <v>44652</v>
+        <v>44682</v>
       </c>
       <c r="B50">
-        <v>1641994</v>
+        <v>1521826</v>
       </c>
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A51" s="1">
-        <v>44621</v>
+        <v>44652</v>
       </c>
       <c r="B51">
-        <v>1472810</v>
+        <v>1641994</v>
       </c>
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A52" s="1">
-        <v>44593</v>
+        <v>44621</v>
       </c>
       <c r="B52">
-        <v>1518238</v>
+        <v>1472810</v>
       </c>
     </row>
     <row r="53" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A53" s="1">
-        <v>44562</v>
+        <v>44593</v>
       </c>
       <c r="B53">
-        <v>1552414</v>
+        <v>1518238</v>
       </c>
     </row>
     <row r="54" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A54" s="1">
-        <v>44531</v>
+        <v>44562</v>
       </c>
       <c r="B54">
-        <v>1583040</v>
+        <v>1552414</v>
       </c>
     </row>
     <row r="55" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A55" s="1">
-        <v>44501</v>
+        <v>44531</v>
       </c>
       <c r="B55">
-        <v>1816879</v>
+        <v>1583040</v>
       </c>
     </row>
     <row r="56" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A56" s="1">
-        <v>44470</v>
+        <v>44501</v>
       </c>
       <c r="B56">
-        <v>1834103</v>
+        <v>1816879</v>
       </c>
     </row>
     <row r="57" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A57" s="1">
-        <v>44440</v>
+        <v>44470</v>
       </c>
       <c r="B57">
-        <v>1746520</v>
+        <v>1834103</v>
       </c>
     </row>
     <row r="58" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A58" s="1">
-        <v>44409</v>
+        <v>44440</v>
       </c>
       <c r="B58">
-        <v>1877773</v>
+        <v>1746520</v>
       </c>
     </row>
     <row r="59" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A59" s="1">
-        <v>44378</v>
+        <v>44409</v>
       </c>
       <c r="B59">
-        <v>1496460</v>
+        <v>1877773</v>
       </c>
     </row>
     <row r="60" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A60" s="1">
-        <v>44348</v>
+        <v>44378</v>
       </c>
       <c r="B60">
-        <v>1613657</v>
+        <v>1496460</v>
       </c>
     </row>
     <row r="61" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A61" s="1">
-        <v>44317</v>
+        <v>44348</v>
       </c>
       <c r="B61">
-        <v>1568943</v>
+        <v>1613657</v>
       </c>
     </row>
     <row r="62" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A62" s="1">
-        <v>44287</v>
+        <v>44317</v>
       </c>
       <c r="B62">
-        <v>1545981</v>
+        <v>1568943</v>
       </c>
     </row>
     <row r="63" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A63" s="1">
-        <v>44256</v>
+        <v>44287</v>
       </c>
       <c r="B63">
-        <v>1445970</v>
+        <v>1545981</v>
       </c>
     </row>
     <row r="64" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A64" s="1">
-        <v>44228</v>
+        <v>44256</v>
       </c>
       <c r="B64">
-        <v>1300808</v>
+        <v>1445970</v>
       </c>
     </row>
     <row r="65" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A65" s="1">
-        <v>44197</v>
+        <v>44228</v>
       </c>
       <c r="B65">
-        <v>1324963</v>
+        <v>1300808</v>
       </c>
     </row>
     <row r="66" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A66" s="1">
-        <v>44166</v>
+        <v>44197</v>
       </c>
       <c r="B66">
-        <v>1265698</v>
+        <v>1324963</v>
       </c>
     </row>
     <row r="67" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A67" s="1">
-        <v>44136</v>
+        <v>44166</v>
       </c>
       <c r="B67">
-        <v>1564505</v>
+        <v>1265698</v>
       </c>
     </row>
     <row r="68" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A68" s="1">
-        <v>44105</v>
+        <v>44136</v>
       </c>
       <c r="B68">
-        <v>1573665</v>
+        <v>1564505</v>
       </c>
     </row>
     <row r="69" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A69" s="1">
-        <v>44075</v>
+        <v>44105</v>
       </c>
       <c r="B69">
-        <v>1722007</v>
+        <v>1573665</v>
       </c>
     </row>
     <row r="70" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A70" s="1">
-        <v>44044</v>
+        <v>44075</v>
       </c>
       <c r="B70">
-        <v>1699106</v>
+        <v>1722007</v>
       </c>
     </row>
     <row r="71" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A71" s="1">
-        <v>44013</v>
+        <v>44044</v>
       </c>
       <c r="B71">
-        <v>1698036</v>
+        <v>1699106</v>
       </c>
     </row>
     <row r="72" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A72" s="1">
-        <v>43983</v>
+        <v>44013</v>
       </c>
       <c r="B72">
-        <v>1898331</v>
+        <v>1698036</v>
       </c>
     </row>
     <row r="73" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A73" s="1">
-        <v>43952</v>
+        <v>43983</v>
       </c>
       <c r="B73">
-        <v>2029579</v>
+        <v>1898331</v>
       </c>
     </row>
     <row r="74" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A74" s="1">
-        <v>43922</v>
+        <v>43952</v>
       </c>
       <c r="B74">
-        <v>2044498</v>
+        <v>2029579</v>
       </c>
     </row>
     <row r="75" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A75" s="1">
-        <v>43891</v>
+        <v>43922</v>
       </c>
       <c r="B75">
-        <v>1729592</v>
+        <v>2044498</v>
       </c>
     </row>
     <row r="76" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A76" s="1">
-        <v>43862</v>
+        <v>43891</v>
       </c>
       <c r="B76">
-        <v>1700261</v>
+        <v>1729592</v>
       </c>
     </row>
     <row r="77" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A77" s="1">
-        <v>43831</v>
+        <v>43862</v>
       </c>
       <c r="B77">
-        <v>1755417</v>
+        <v>1700261</v>
       </c>
     </row>
     <row r="78" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A78" s="1">
-        <v>43800</v>
+        <v>43831</v>
       </c>
       <c r="B78">
-        <v>2007124</v>
+        <v>1755417</v>
       </c>
     </row>
     <row r="79" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A79" s="1">
-        <v>43770</v>
+        <v>43800</v>
       </c>
       <c r="B79">
-        <v>2255035</v>
+        <v>2007124</v>
       </c>
     </row>
     <row r="80" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A80" s="1">
-        <v>43739</v>
+        <v>43770</v>
       </c>
       <c r="B80">
-        <v>2351994</v>
+        <v>2255035</v>
       </c>
     </row>
     <row r="81" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A81" s="1">
-        <v>43709</v>
+        <v>43739</v>
       </c>
       <c r="B81">
-        <v>2448272</v>
+        <v>2351994</v>
       </c>
     </row>
     <row r="82" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A82" s="1">
-        <v>43678</v>
+        <v>43709</v>
       </c>
       <c r="B82">
-        <v>2251831</v>
+        <v>2448272</v>
       </c>
     </row>
     <row r="83" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A83" s="1">
-        <v>43647</v>
+        <v>43678</v>
       </c>
       <c r="B83">
-        <v>2378099</v>
+        <v>2251831</v>
       </c>
     </row>
     <row r="84" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A84" s="1">
-        <v>43617</v>
+        <v>43647</v>
       </c>
       <c r="B84">
-        <v>2410746</v>
+        <v>2378099</v>
       </c>
     </row>
     <row r="85" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A85" s="1">
-        <v>43586</v>
+        <v>43617</v>
       </c>
       <c r="B85">
-        <v>2447250</v>
+        <v>2410746</v>
       </c>
     </row>
     <row r="86" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A86" s="1">
-        <v>43556</v>
+        <v>43586</v>
       </c>
       <c r="B86">
-        <v>2729389</v>
+        <v>2447250</v>
       </c>
     </row>
     <row r="87" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A87" s="1">
-        <v>43525</v>
+        <v>43556</v>
       </c>
       <c r="B87">
-        <v>2922852</v>
+        <v>2729389</v>
       </c>
     </row>
     <row r="88" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A88" s="1">
-        <v>43497</v>
+        <v>43525</v>
       </c>
       <c r="B88">
-        <v>3059400</v>
+        <v>2922852</v>
       </c>
     </row>
     <row r="89" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A89" s="1">
-        <v>43466</v>
+        <v>43497</v>
       </c>
       <c r="B89">
-        <v>3005313</v>
+        <v>3059400</v>
       </c>
     </row>
     <row r="90" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A90" s="1">
-        <v>43435</v>
+        <v>43466</v>
       </c>
       <c r="B90">
-        <v>3215052</v>
+        <v>3005313</v>
       </c>
     </row>
     <row r="91" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A91" s="1">
-        <v>43405</v>
+        <v>43435</v>
       </c>
       <c r="B91">
-        <v>3007086</v>
+        <v>3215052</v>
       </c>
     </row>
     <row r="92" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A92" s="1">
-        <v>43374</v>
+        <v>43405</v>
       </c>
       <c r="B92">
-        <v>2722478</v>
+        <v>3007086</v>
       </c>
     </row>
     <row r="93" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A93" s="1">
-        <v>43344</v>
+        <v>43374</v>
       </c>
       <c r="B93">
-        <v>2529447</v>
+        <v>2722478</v>
       </c>
     </row>
     <row r="94" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A94" s="1">
-        <v>43313</v>
+        <v>43344</v>
       </c>
       <c r="B94">
-        <v>2054915</v>
+        <v>2529447</v>
       </c>
     </row>
     <row r="95" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A95" s="1">
-        <v>43282</v>
+        <v>43313</v>
       </c>
       <c r="B95">
-        <v>2214689</v>
+        <v>2054915</v>
       </c>
     </row>
     <row r="96" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A96" s="1">
-        <v>43252</v>
+        <v>43282</v>
       </c>
       <c r="B96">
-        <v>2188660</v>
+        <v>2214689</v>
       </c>
     </row>
     <row r="97" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A97" s="1">
-        <v>43221</v>
+        <v>43252</v>
       </c>
       <c r="B97">
-        <v>2170431</v>
+        <v>2188660</v>
       </c>
     </row>
     <row r="98" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A98" s="1">
-        <v>43191</v>
+        <v>43221</v>
       </c>
       <c r="B98">
-        <v>2181478</v>
+        <v>2170431</v>
       </c>
     </row>
     <row r="99" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A99" s="1">
-        <v>43160</v>
+        <v>43191</v>
       </c>
       <c r="B99">
-        <v>2323458</v>
+        <v>2181478</v>
       </c>
     </row>
     <row r="100" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A100" s="1">
-        <v>43132</v>
+        <v>43160</v>
       </c>
       <c r="B100">
-        <v>2478186</v>
+        <v>2323458</v>
       </c>
     </row>
     <row r="101" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A101" s="1">
-        <v>43101</v>
+        <v>43132</v>
       </c>
       <c r="B101">
-        <v>2547680</v>
+        <v>2478186</v>
       </c>
     </row>
     <row r="102" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A102" s="1">
-        <v>43070</v>
+        <v>43101</v>
       </c>
       <c r="B102">
-        <v>2732093</v>
+        <v>2547680</v>
       </c>
     </row>
     <row r="103" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A103" s="1">
-        <v>43040</v>
+        <v>43070</v>
       </c>
       <c r="B103">
-        <v>2553739</v>
+        <v>2732093</v>
       </c>
     </row>
     <row r="104" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A104" s="1">
-        <v>43009</v>
+        <v>43040</v>
       </c>
       <c r="B104">
-        <v>2203383</v>
+        <v>2553739</v>
       </c>
     </row>
     <row r="105" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A105" s="1">
-        <v>42979</v>
+        <v>43009</v>
       </c>
       <c r="B105">
-        <v>2020505</v>
+        <v>2203383</v>
       </c>
     </row>
     <row r="106" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A106" s="1">
-        <v>42948</v>
+        <v>42979</v>
       </c>
       <c r="B106">
-        <v>1942001</v>
+        <v>2020505</v>
       </c>
     </row>
     <row r="107" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A107" s="1">
-        <v>42917</v>
+        <v>42948</v>
       </c>
       <c r="B107">
-        <v>1785082</v>
+        <v>1942001</v>
       </c>
     </row>
     <row r="108" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A108" s="1">
-        <v>42887</v>
+        <v>42917</v>
       </c>
       <c r="B108">
-        <v>1527071</v>
+        <v>1785082</v>
       </c>
     </row>
     <row r="109" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A109" s="1">
-        <v>42856</v>
+        <v>42887</v>
       </c>
       <c r="B109">
-        <v>1557354</v>
+        <v>1527071</v>
       </c>
     </row>
     <row r="110" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A110" s="1">
-        <v>42826</v>
+        <v>42856</v>
       </c>
       <c r="B110">
-        <v>599894</v>
+        <v>1557354</v>
       </c>
     </row>
     <row r="111" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A111" s="1">
-        <v>42795</v>
+        <v>42826</v>
       </c>
       <c r="B111">
-        <v>1552988</v>
+        <v>599894</v>
       </c>
     </row>
     <row r="112" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A112" s="1">
-        <v>42767</v>
+        <v>42795</v>
       </c>
       <c r="B112">
-        <v>1459265</v>
+        <v>1552988</v>
       </c>
     </row>
     <row r="113" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A113" s="1">
-        <v>42736</v>
+        <v>42767</v>
       </c>
       <c r="B113">
-        <v>1541082</v>
+        <v>1459265</v>
       </c>
     </row>
     <row r="114" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A114" s="1">
-        <v>42705</v>
+        <v>42736</v>
       </c>
       <c r="B114">
-        <v>1665388</v>
+        <v>1541082</v>
       </c>
     </row>
     <row r="115" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A115" s="1">
-        <v>42675</v>
+        <v>42705</v>
       </c>
       <c r="B115">
-        <v>1662811</v>
+        <v>1665388</v>
       </c>
     </row>
     <row r="116" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A116" s="1">
-        <v>42644</v>
+        <v>42675</v>
       </c>
       <c r="B116">
-        <v>1574288</v>
+        <v>1662811</v>
       </c>
     </row>
     <row r="117" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A117" s="1">
-        <v>42614</v>
+        <v>42644</v>
       </c>
       <c r="B117">
-        <v>1546413</v>
+        <v>1574288</v>
       </c>
     </row>
     <row r="118" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A118" s="1">
-        <v>42583</v>
+        <v>42614</v>
       </c>
       <c r="B118">
-        <v>1464080</v>
+        <v>1546413</v>
       </c>
     </row>
     <row r="119" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A119" s="1">
-        <v>42552</v>
+        <v>42583</v>
       </c>
       <c r="B119">
-        <v>1770083</v>
+        <v>1464080</v>
       </c>
     </row>
     <row r="120" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A120" s="1">
-        <v>42522</v>
+        <v>42552</v>
       </c>
       <c r="B120">
-        <v>1774624</v>
+        <v>1770083</v>
       </c>
     </row>
     <row r="121" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A121" s="1">
-        <v>42491</v>
+        <v>42522</v>
       </c>
       <c r="B121">
-        <v>1649858</v>
+        <v>1774624</v>
       </c>
     </row>
     <row r="122" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A122" s="1">
-        <v>42461</v>
+        <v>42491</v>
       </c>
       <c r="B122">
-        <v>1803894</v>
+        <v>1649858</v>
       </c>
     </row>
     <row r="123" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A123" s="1">
-        <v>42430</v>
+        <v>42461</v>
       </c>
       <c r="B123">
-        <v>1885630</v>
+        <v>1803894</v>
       </c>
     </row>
     <row r="124" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A124" s="1">
-        <v>42401</v>
+        <v>42430</v>
       </c>
       <c r="B124">
-        <v>2170341</v>
+        <v>1885630</v>
       </c>
     </row>
     <row r="125" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A125" s="1">
+        <v>42401</v>
+      </c>
+      <c r="B125">
+        <v>2170341</v>
+      </c>
+    </row>
+    <row r="126" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A126" s="1">
         <v>42370</v>
       </c>
-      <c r="B125">
+      <c r="B126">
         <v>2308582</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A5:B41 A1:B2" numberStoredAsText="1"/>
+    <ignoredError sqref="A6:B42 A1:B2" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: add Shape Calendar research artifact + new term structure data (2008-2017)
Build standalone FCPO_Shape_Calendar with per-year calendar pages and
cross-year summary showing seasonal shape distribution patterns.
Added historical term structure CSVs (2008-2017) and updated 2026-2027 data.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Raw Data/Stock and Production/FCPO Stock 3Y.xlsx
+++ b/Raw Data/Stock and Production/FCPO Stock 3Y.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ClaudeCode\Raw Data\Stock and Production\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{601910F9-B5DD-4732-ABAE-4E01B784015A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B67416D-4751-4B53-B5E8-4BEADD5667B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="39390" yWindow="-20835" windowWidth="28800" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-38520" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Table Data" sheetId="1" r:id="rId1"/>
@@ -412,7 +412,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B126"/>
+  <dimension ref="A1:B127"/>
   <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.875" customWidth="1"/>
@@ -437,1000 +437,1008 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
-        <v>46113</v>
+        <v>46143</v>
       </c>
       <c r="B3">
-        <v>2309474</v>
+        <v>2427835</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
-        <v>46082</v>
+        <v>46113</v>
       </c>
       <c r="B4">
-        <v>2270574</v>
+        <v>2309474</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
-        <v>46054</v>
+        <v>46082</v>
       </c>
       <c r="B5">
-        <v>2704286</v>
+        <v>2270574</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
-        <v>46023</v>
+        <v>46054</v>
       </c>
       <c r="B6">
-        <v>2815493</v>
+        <v>2704286</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
-        <v>45992</v>
+        <v>46023</v>
       </c>
       <c r="B7">
-        <v>3051147</v>
+        <v>2815493</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
-        <v>45962</v>
+        <v>45992</v>
       </c>
       <c r="B8">
-        <v>2835578</v>
+        <v>3051147</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
-        <v>45931</v>
+        <v>45962</v>
       </c>
       <c r="B9">
-        <v>2508396</v>
+        <v>2835578</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
-        <v>45901</v>
+        <v>45931</v>
       </c>
       <c r="B10">
-        <v>2359572</v>
+        <v>2508396</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
-        <v>45870</v>
+        <v>45901</v>
       </c>
       <c r="B11">
-        <v>2202413</v>
+        <v>2359572</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
-        <v>45839</v>
+        <v>45870</v>
       </c>
       <c r="B12">
-        <v>2114085</v>
+        <v>2202413</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
-        <v>45809</v>
+        <v>45839</v>
       </c>
       <c r="B13">
-        <v>2031560</v>
+        <v>2114085</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
-        <v>45778</v>
+        <v>45809</v>
       </c>
       <c r="B14">
-        <v>1982759</v>
+        <v>2031560</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="1">
-        <v>45748</v>
+        <v>45778</v>
       </c>
       <c r="B15">
-        <v>1866124</v>
+        <v>1982759</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" s="1">
-        <v>45717</v>
+        <v>45748</v>
       </c>
       <c r="B16">
-        <v>1562817</v>
+        <v>1866124</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="1">
-        <v>45689</v>
+        <v>45717</v>
       </c>
       <c r="B17">
-        <v>1509525</v>
+        <v>1562817</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" s="1">
-        <v>45658</v>
+        <v>45689</v>
       </c>
       <c r="B18">
-        <v>1580252</v>
+        <v>1509525</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" s="1">
-        <v>45627</v>
+        <v>45658</v>
       </c>
       <c r="B19">
-        <v>1708756</v>
+        <v>1580252</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" s="1">
-        <v>45597</v>
+        <v>45627</v>
       </c>
       <c r="B20">
-        <v>1835641</v>
+        <v>1708756</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" s="1">
-        <v>45566</v>
+        <v>45597</v>
       </c>
       <c r="B21">
-        <v>1885183</v>
+        <v>1835641</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" s="1">
-        <v>45536</v>
+        <v>45566</v>
       </c>
       <c r="B22">
-        <v>2011768</v>
+        <v>1885183</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" s="1">
-        <v>45505</v>
+        <v>45536</v>
       </c>
       <c r="B23">
-        <v>1883328</v>
+        <v>2011768</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" s="1">
-        <v>45474</v>
+        <v>45505</v>
       </c>
       <c r="B24">
-        <v>1754384</v>
+        <v>1883328</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" s="1">
-        <v>45444</v>
+        <v>45474</v>
       </c>
       <c r="B25">
-        <v>1831239</v>
+        <v>1754384</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" s="1">
-        <v>45413</v>
+        <v>45444</v>
       </c>
       <c r="B26">
-        <v>1753211</v>
+        <v>1831239</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" s="1">
-        <v>45383</v>
+        <v>45413</v>
       </c>
       <c r="B27">
-        <v>1744459</v>
+        <v>1753211</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" s="1">
-        <v>45352</v>
+        <v>45383</v>
       </c>
       <c r="B28">
-        <v>1714973</v>
+        <v>1744459</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" s="1">
-        <v>45323</v>
+        <v>45352</v>
       </c>
       <c r="B29">
-        <v>1919210</v>
+        <v>1714973</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" s="1">
-        <v>45292</v>
+        <v>45323</v>
       </c>
       <c r="B30">
-        <v>2019781</v>
+        <v>1919210</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31" s="1">
-        <v>45261</v>
+        <v>45292</v>
       </c>
       <c r="B31">
-        <v>2291167</v>
+        <v>2019781</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32" s="1">
-        <v>45231</v>
+        <v>45261</v>
       </c>
       <c r="B32">
-        <v>2420398</v>
+        <v>2291167</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" s="1">
-        <v>45200</v>
+        <v>45231</v>
       </c>
       <c r="B33">
-        <v>2448852</v>
+        <v>2420398</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" s="1">
-        <v>45170</v>
+        <v>45200</v>
       </c>
       <c r="B34">
-        <v>2313569</v>
+        <v>2448852</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" s="1">
-        <v>45139</v>
+        <v>45170</v>
       </c>
       <c r="B35">
-        <v>2110980</v>
+        <v>2313569</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36" s="1">
-        <v>45108</v>
+        <v>45139</v>
       </c>
       <c r="B36">
-        <v>1734157</v>
+        <v>2110980</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37" s="1">
-        <v>45078</v>
+        <v>45108</v>
       </c>
       <c r="B37">
-        <v>1720567</v>
+        <v>1734157</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38" s="1">
-        <v>45047</v>
+        <v>45078</v>
       </c>
       <c r="B38">
-        <v>1686782</v>
+        <v>1720567</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" s="1">
-        <v>45017</v>
+        <v>45047</v>
       </c>
       <c r="B39">
-        <v>1497617</v>
+        <v>1686782</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" s="1">
-        <v>44986</v>
+        <v>45017</v>
       </c>
       <c r="B40">
-        <v>1674022</v>
+        <v>1497617</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41" s="1">
-        <v>44958</v>
+        <v>44986</v>
       </c>
       <c r="B41">
-        <v>2119848</v>
+        <v>1674022</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A42" s="1">
-        <v>44927</v>
+        <v>44958</v>
       </c>
       <c r="B42">
-        <v>2268198</v>
+        <v>2119848</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A43" s="1">
-        <v>44896</v>
+        <v>44927</v>
       </c>
       <c r="B43">
-        <v>2196574</v>
+        <v>2268198</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A44" s="1">
-        <v>44866</v>
+        <v>44896</v>
       </c>
       <c r="B44">
-        <v>2288471</v>
+        <v>2196574</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A45" s="1">
-        <v>44835</v>
+        <v>44866</v>
       </c>
       <c r="B45">
-        <v>2408293</v>
+        <v>2288471</v>
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A46" s="1">
-        <v>44805</v>
+        <v>44835</v>
       </c>
       <c r="B46">
-        <v>2317020</v>
+        <v>2408293</v>
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A47" s="1">
-        <v>44774</v>
+        <v>44805</v>
       </c>
       <c r="B47">
-        <v>2094667</v>
+        <v>2317020</v>
       </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A48" s="1">
-        <v>44743</v>
+        <v>44774</v>
       </c>
       <c r="B48">
-        <v>1772804</v>
+        <v>2094667</v>
       </c>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A49" s="1">
-        <v>44713</v>
+        <v>44743</v>
       </c>
       <c r="B49">
-        <v>1645831</v>
+        <v>1772804</v>
       </c>
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A50" s="1">
-        <v>44682</v>
+        <v>44713</v>
       </c>
       <c r="B50">
-        <v>1521826</v>
+        <v>1645831</v>
       </c>
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A51" s="1">
-        <v>44652</v>
+        <v>44682</v>
       </c>
       <c r="B51">
-        <v>1641994</v>
+        <v>1521826</v>
       </c>
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A52" s="1">
-        <v>44621</v>
+        <v>44652</v>
       </c>
       <c r="B52">
-        <v>1472810</v>
+        <v>1641994</v>
       </c>
     </row>
     <row r="53" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A53" s="1">
-        <v>44593</v>
+        <v>44621</v>
       </c>
       <c r="B53">
-        <v>1518238</v>
+        <v>1472810</v>
       </c>
     </row>
     <row r="54" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A54" s="1">
-        <v>44562</v>
+        <v>44593</v>
       </c>
       <c r="B54">
-        <v>1552414</v>
+        <v>1518238</v>
       </c>
     </row>
     <row r="55" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A55" s="1">
-        <v>44531</v>
+        <v>44562</v>
       </c>
       <c r="B55">
-        <v>1583040</v>
+        <v>1552414</v>
       </c>
     </row>
     <row r="56" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A56" s="1">
-        <v>44501</v>
+        <v>44531</v>
       </c>
       <c r="B56">
-        <v>1816879</v>
+        <v>1583040</v>
       </c>
     </row>
     <row r="57" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A57" s="1">
-        <v>44470</v>
+        <v>44501</v>
       </c>
       <c r="B57">
-        <v>1834103</v>
+        <v>1816879</v>
       </c>
     </row>
     <row r="58" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A58" s="1">
-        <v>44440</v>
+        <v>44470</v>
       </c>
       <c r="B58">
-        <v>1746520</v>
+        <v>1834103</v>
       </c>
     </row>
     <row r="59" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A59" s="1">
-        <v>44409</v>
+        <v>44440</v>
       </c>
       <c r="B59">
-        <v>1877773</v>
+        <v>1746520</v>
       </c>
     </row>
     <row r="60" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A60" s="1">
-        <v>44378</v>
+        <v>44409</v>
       </c>
       <c r="B60">
-        <v>1496460</v>
+        <v>1877773</v>
       </c>
     </row>
     <row r="61" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A61" s="1">
-        <v>44348</v>
+        <v>44378</v>
       </c>
       <c r="B61">
-        <v>1613657</v>
+        <v>1496460</v>
       </c>
     </row>
     <row r="62" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A62" s="1">
-        <v>44317</v>
+        <v>44348</v>
       </c>
       <c r="B62">
-        <v>1568943</v>
+        <v>1613657</v>
       </c>
     </row>
     <row r="63" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A63" s="1">
-        <v>44287</v>
+        <v>44317</v>
       </c>
       <c r="B63">
-        <v>1545981</v>
+        <v>1568943</v>
       </c>
     </row>
     <row r="64" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A64" s="1">
-        <v>44256</v>
+        <v>44287</v>
       </c>
       <c r="B64">
-        <v>1445970</v>
+        <v>1545981</v>
       </c>
     </row>
     <row r="65" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A65" s="1">
-        <v>44228</v>
+        <v>44256</v>
       </c>
       <c r="B65">
-        <v>1300808</v>
+        <v>1445970</v>
       </c>
     </row>
     <row r="66" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A66" s="1">
-        <v>44197</v>
+        <v>44228</v>
       </c>
       <c r="B66">
-        <v>1324963</v>
+        <v>1300808</v>
       </c>
     </row>
     <row r="67" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A67" s="1">
-        <v>44166</v>
+        <v>44197</v>
       </c>
       <c r="B67">
-        <v>1265698</v>
+        <v>1324963</v>
       </c>
     </row>
     <row r="68" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A68" s="1">
-        <v>44136</v>
+        <v>44166</v>
       </c>
       <c r="B68">
-        <v>1564505</v>
+        <v>1265698</v>
       </c>
     </row>
     <row r="69" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A69" s="1">
-        <v>44105</v>
+        <v>44136</v>
       </c>
       <c r="B69">
-        <v>1573665</v>
+        <v>1564505</v>
       </c>
     </row>
     <row r="70" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A70" s="1">
-        <v>44075</v>
+        <v>44105</v>
       </c>
       <c r="B70">
-        <v>1722007</v>
+        <v>1573665</v>
       </c>
     </row>
     <row r="71" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A71" s="1">
-        <v>44044</v>
+        <v>44075</v>
       </c>
       <c r="B71">
-        <v>1699106</v>
+        <v>1722007</v>
       </c>
     </row>
     <row r="72" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A72" s="1">
-        <v>44013</v>
+        <v>44044</v>
       </c>
       <c r="B72">
-        <v>1698036</v>
+        <v>1699106</v>
       </c>
     </row>
     <row r="73" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A73" s="1">
-        <v>43983</v>
+        <v>44013</v>
       </c>
       <c r="B73">
-        <v>1898331</v>
+        <v>1698036</v>
       </c>
     </row>
     <row r="74" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A74" s="1">
-        <v>43952</v>
+        <v>43983</v>
       </c>
       <c r="B74">
-        <v>2029579</v>
+        <v>1898331</v>
       </c>
     </row>
     <row r="75" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A75" s="1">
-        <v>43922</v>
+        <v>43952</v>
       </c>
       <c r="B75">
-        <v>2044498</v>
+        <v>2029579</v>
       </c>
     </row>
     <row r="76" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A76" s="1">
-        <v>43891</v>
+        <v>43922</v>
       </c>
       <c r="B76">
-        <v>1729592</v>
+        <v>2044498</v>
       </c>
     </row>
     <row r="77" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A77" s="1">
-        <v>43862</v>
+        <v>43891</v>
       </c>
       <c r="B77">
-        <v>1700261</v>
+        <v>1729592</v>
       </c>
     </row>
     <row r="78" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A78" s="1">
-        <v>43831</v>
+        <v>43862</v>
       </c>
       <c r="B78">
-        <v>1755417</v>
+        <v>1700261</v>
       </c>
     </row>
     <row r="79" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A79" s="1">
-        <v>43800</v>
+        <v>43831</v>
       </c>
       <c r="B79">
-        <v>2007124</v>
+        <v>1755417</v>
       </c>
     </row>
     <row r="80" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A80" s="1">
-        <v>43770</v>
+        <v>43800</v>
       </c>
       <c r="B80">
-        <v>2255035</v>
+        <v>2007124</v>
       </c>
     </row>
     <row r="81" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A81" s="1">
-        <v>43739</v>
+        <v>43770</v>
       </c>
       <c r="B81">
-        <v>2351994</v>
+        <v>2255035</v>
       </c>
     </row>
     <row r="82" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A82" s="1">
-        <v>43709</v>
+        <v>43739</v>
       </c>
       <c r="B82">
-        <v>2448272</v>
+        <v>2351994</v>
       </c>
     </row>
     <row r="83" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A83" s="1">
-        <v>43678</v>
+        <v>43709</v>
       </c>
       <c r="B83">
-        <v>2251831</v>
+        <v>2448272</v>
       </c>
     </row>
     <row r="84" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A84" s="1">
-        <v>43647</v>
+        <v>43678</v>
       </c>
       <c r="B84">
-        <v>2378099</v>
+        <v>2251831</v>
       </c>
     </row>
     <row r="85" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A85" s="1">
-        <v>43617</v>
+        <v>43647</v>
       </c>
       <c r="B85">
-        <v>2410746</v>
+        <v>2378099</v>
       </c>
     </row>
     <row r="86" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A86" s="1">
-        <v>43586</v>
+        <v>43617</v>
       </c>
       <c r="B86">
-        <v>2447250</v>
+        <v>2410746</v>
       </c>
     </row>
     <row r="87" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A87" s="1">
-        <v>43556</v>
+        <v>43586</v>
       </c>
       <c r="B87">
-        <v>2729389</v>
+        <v>2447250</v>
       </c>
     </row>
     <row r="88" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A88" s="1">
-        <v>43525</v>
+        <v>43556</v>
       </c>
       <c r="B88">
-        <v>2922852</v>
+        <v>2729389</v>
       </c>
     </row>
     <row r="89" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A89" s="1">
-        <v>43497</v>
+        <v>43525</v>
       </c>
       <c r="B89">
-        <v>3059400</v>
+        <v>2922852</v>
       </c>
     </row>
     <row r="90" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A90" s="1">
-        <v>43466</v>
+        <v>43497</v>
       </c>
       <c r="B90">
-        <v>3005313</v>
+        <v>3059400</v>
       </c>
     </row>
     <row r="91" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A91" s="1">
-        <v>43435</v>
+        <v>43466</v>
       </c>
       <c r="B91">
-        <v>3215052</v>
+        <v>3005313</v>
       </c>
     </row>
     <row r="92" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A92" s="1">
-        <v>43405</v>
+        <v>43435</v>
       </c>
       <c r="B92">
-        <v>3007086</v>
+        <v>3215052</v>
       </c>
     </row>
     <row r="93" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A93" s="1">
-        <v>43374</v>
+        <v>43405</v>
       </c>
       <c r="B93">
-        <v>2722478</v>
+        <v>3007086</v>
       </c>
     </row>
     <row r="94" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A94" s="1">
-        <v>43344</v>
+        <v>43374</v>
       </c>
       <c r="B94">
-        <v>2529447</v>
+        <v>2722478</v>
       </c>
     </row>
     <row r="95" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A95" s="1">
-        <v>43313</v>
+        <v>43344</v>
       </c>
       <c r="B95">
-        <v>2054915</v>
+        <v>2529447</v>
       </c>
     </row>
     <row r="96" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A96" s="1">
-        <v>43282</v>
+        <v>43313</v>
       </c>
       <c r="B96">
-        <v>2214689</v>
+        <v>2054915</v>
       </c>
     </row>
     <row r="97" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A97" s="1">
-        <v>43252</v>
+        <v>43282</v>
       </c>
       <c r="B97">
-        <v>2188660</v>
+        <v>2214689</v>
       </c>
     </row>
     <row r="98" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A98" s="1">
-        <v>43221</v>
+        <v>43252</v>
       </c>
       <c r="B98">
-        <v>2170431</v>
+        <v>2188660</v>
       </c>
     </row>
     <row r="99" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A99" s="1">
-        <v>43191</v>
+        <v>43221</v>
       </c>
       <c r="B99">
-        <v>2181478</v>
+        <v>2170431</v>
       </c>
     </row>
     <row r="100" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A100" s="1">
-        <v>43160</v>
+        <v>43191</v>
       </c>
       <c r="B100">
-        <v>2323458</v>
+        <v>2181478</v>
       </c>
     </row>
     <row r="101" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A101" s="1">
-        <v>43132</v>
+        <v>43160</v>
       </c>
       <c r="B101">
-        <v>2478186</v>
+        <v>2323458</v>
       </c>
     </row>
     <row r="102" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A102" s="1">
-        <v>43101</v>
+        <v>43132</v>
       </c>
       <c r="B102">
-        <v>2547680</v>
+        <v>2478186</v>
       </c>
     </row>
     <row r="103" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A103" s="1">
-        <v>43070</v>
+        <v>43101</v>
       </c>
       <c r="B103">
-        <v>2732093</v>
+        <v>2547680</v>
       </c>
     </row>
     <row r="104" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A104" s="1">
-        <v>43040</v>
+        <v>43070</v>
       </c>
       <c r="B104">
-        <v>2553739</v>
+        <v>2732093</v>
       </c>
     </row>
     <row r="105" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A105" s="1">
-        <v>43009</v>
+        <v>43040</v>
       </c>
       <c r="B105">
-        <v>2203383</v>
+        <v>2553739</v>
       </c>
     </row>
     <row r="106" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A106" s="1">
-        <v>42979</v>
+        <v>43009</v>
       </c>
       <c r="B106">
-        <v>2020505</v>
+        <v>2203383</v>
       </c>
     </row>
     <row r="107" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A107" s="1">
-        <v>42948</v>
+        <v>42979</v>
       </c>
       <c r="B107">
-        <v>1942001</v>
+        <v>2020505</v>
       </c>
     </row>
     <row r="108" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A108" s="1">
-        <v>42917</v>
+        <v>42948</v>
       </c>
       <c r="B108">
-        <v>1785082</v>
+        <v>1942001</v>
       </c>
     </row>
     <row r="109" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A109" s="1">
-        <v>42887</v>
+        <v>42917</v>
       </c>
       <c r="B109">
-        <v>1527071</v>
+        <v>1785082</v>
       </c>
     </row>
     <row r="110" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A110" s="1">
-        <v>42856</v>
+        <v>42887</v>
       </c>
       <c r="B110">
-        <v>1557354</v>
+        <v>1527071</v>
       </c>
     </row>
     <row r="111" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A111" s="1">
-        <v>42826</v>
+        <v>42856</v>
       </c>
       <c r="B111">
-        <v>599894</v>
+        <v>1557354</v>
       </c>
     </row>
     <row r="112" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A112" s="1">
-        <v>42795</v>
+        <v>42826</v>
       </c>
       <c r="B112">
-        <v>1552988</v>
+        <v>599894</v>
       </c>
     </row>
     <row r="113" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A113" s="1">
-        <v>42767</v>
+        <v>42795</v>
       </c>
       <c r="B113">
-        <v>1459265</v>
+        <v>1552988</v>
       </c>
     </row>
     <row r="114" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A114" s="1">
-        <v>42736</v>
+        <v>42767</v>
       </c>
       <c r="B114">
-        <v>1541082</v>
+        <v>1459265</v>
       </c>
     </row>
     <row r="115" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A115" s="1">
-        <v>42705</v>
+        <v>42736</v>
       </c>
       <c r="B115">
-        <v>1665388</v>
+        <v>1541082</v>
       </c>
     </row>
     <row r="116" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A116" s="1">
-        <v>42675</v>
+        <v>42705</v>
       </c>
       <c r="B116">
-        <v>1662811</v>
+        <v>1665388</v>
       </c>
     </row>
     <row r="117" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A117" s="1">
-        <v>42644</v>
+        <v>42675</v>
       </c>
       <c r="B117">
-        <v>1574288</v>
+        <v>1662811</v>
       </c>
     </row>
     <row r="118" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A118" s="1">
-        <v>42614</v>
+        <v>42644</v>
       </c>
       <c r="B118">
-        <v>1546413</v>
+        <v>1574288</v>
       </c>
     </row>
     <row r="119" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A119" s="1">
-        <v>42583</v>
+        <v>42614</v>
       </c>
       <c r="B119">
-        <v>1464080</v>
+        <v>1546413</v>
       </c>
     </row>
     <row r="120" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A120" s="1">
-        <v>42552</v>
+        <v>42583</v>
       </c>
       <c r="B120">
-        <v>1770083</v>
+        <v>1464080</v>
       </c>
     </row>
     <row r="121" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A121" s="1">
-        <v>42522</v>
+        <v>42552</v>
       </c>
       <c r="B121">
-        <v>1774624</v>
+        <v>1770083</v>
       </c>
     </row>
     <row r="122" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A122" s="1">
-        <v>42491</v>
+        <v>42522</v>
       </c>
       <c r="B122">
-        <v>1649858</v>
+        <v>1774624</v>
       </c>
     </row>
     <row r="123" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A123" s="1">
-        <v>42461</v>
+        <v>42491</v>
       </c>
       <c r="B123">
-        <v>1803894</v>
+        <v>1649858</v>
       </c>
     </row>
     <row r="124" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A124" s="1">
-        <v>42430</v>
+        <v>42461</v>
       </c>
       <c r="B124">
-        <v>1885630</v>
+        <v>1803894</v>
       </c>
     </row>
     <row r="125" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A125" s="1">
-        <v>42401</v>
+        <v>42430</v>
       </c>
       <c r="B125">
-        <v>2170341</v>
+        <v>1885630</v>
       </c>
     </row>
     <row r="126" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A126" s="1">
+        <v>42401</v>
+      </c>
+      <c r="B126">
+        <v>2170341</v>
+      </c>
+    </row>
+    <row r="127" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A127" s="1">
         <v>42370</v>
       </c>
-      <c r="B126">
+      <c r="B127">
         <v>2308582</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A6:B42 A1:B2" numberStoredAsText="1"/>
+    <ignoredError sqref="A7:B43 A1:B2" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>